<commit_message>
Update leads tracker 2026-09-02
</commit_message>
<xml_diff>
--- a/leads_tracker.xlsx
+++ b/leads_tracker.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -616,6 +616,288 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Fraser River Tunnel Project (George Massey Replacement) — Re-Tender for Major Construction</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Surrey Now-Leader / BC Ministry of Transportation and Infrastructure</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://surreynowleader.com/2026/06/15/b-c-moves-to-re-tender-construction-of-george-massey-tunnel-replacement/</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Pre-position with BC MoTI's Transportation Infrastructure Contracting branch; register on BC Bid and MoTI prequalification now; monitor the EAO project page for the environmental assessment certificate decision expected Q4 2026 — that will trigger the new RFQ/RFP release.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>BC MoTI cancelled its agreement with Cross Fraser Partnership and is re-tendering the $4.15B, eight-lane immersed-tube tunnel replacement; major construction is anticipated to begin in 2027 pending an EAO certificate expected by end of 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Yellowhead Copper Mine (Trekor Metals) — Infrastructure &amp; Civil Engineering Work Package</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Mining Weekly / BC Gov News / Trekor Metals</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://www.miningweekly.com/article/yellowhead-copper-project-canada-update-2026-07-10</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Contact Trekor's project team in Barriere, BC via the Yellowhead Project community office; monitor the BC EAO EPIC website for the Process Planning phase posting; begin assembling a civil/structural engineering team and Indigenous partnership credentials ahead of an RFQ that could post in late 2026 or early 2027.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Trekor's proposed 90,000-t/d open-pit copper mine northeast of Kamloops received a positive BC EAO Readiness Decision on July 30, 2026 and is advancing through process planning; the two-to-three-year construction phase is projected to support ~8,800 jobs and engineering/site investigation work is underway in summer 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Canagold New Polaris Gold-Antimony Mine — Construction &amp; Engineering Services</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Newsfile Corp / BC Gov News (Look West update)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://www.newsfilecorp.com/release/295407/Canagold-New-Polaris-GoldAntimony-Project-Recognized-as-a-Priority-Project-by-British-Columbia</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Reach out directly to CEO Catalin Kilofliski (catalin@canagoldresources.com / 604-685-9700) to introduce civil, structural, and northern-logistics capabilities; monitor the BC EAO EPIC project page for scoping decisions and pre-qualification notices expected once EA review begins.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Canagold filed its EA application with BC EAO in April 2026 and was added to BC's priority major projects list in May 2026; the $757M underground mine in northwest BC (near Atlin) is advancing through feasibility and permitting, with drilling underway in summer 2026, signalling construction-phase services contracts on the 1–3 year horizon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BC Hydro Grid-Scale Battery Energy Storage System (BESS) — Request for Supplier Qualifications</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BC Hydro / T-Net News</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://www.bchydro.com/work-with-us/selling-clean-energy/grid-scale-battery.html</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Submit RFSQ response before September 16, 2026 — download documents directly from BC Hydro's grid-scale battery procurement page; confirm BC Bid account registration (bcbid.gov.bc.ca) is active; form or confirm civil/structural and electrical design-build partnerships before the RFP stage.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>BC Hydro issued an RFSQ on July 30, 2026 for BC's first grid-scale BESS project (≥100 MW) to be located adjacent to the Vancouver Island Terminal Substation near Duncan; the RFSQ closes September 16, 2026, after which shortlisted firms will be invited to a full RFP process later in 2026 for design, construction, and potentially long-term maintenance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Metro Vancouver Iona Island Wastewater Treatment Plant — Standby Power System Facility</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Metro Vancouver Bids &amp; Tenders / TendersOnTime</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://metrovancouver.bidsandtenders.ca/</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Register immediately on metrovancouver.bidsandtenders.ca and select civil/construction commodity codes to receive live addenda alerts; review the Iona Island procurement timeline page (metrovancouver.org/services/liquid-waste/procurement) for related upcoming RFPs across the Early Works program.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Metro Vancouver posted a construction tender for the Standby Power System Facility for the Iona Island WWTP Projects, part of the multi-billion-dollar federally mandated secondary-treatment upgrade program; bids posted on the Metro Vancouver bids-and-tenders platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Federal Airports Capital Assistance Program — Six BC Airport Infrastructure Projects ($23.5M)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Transport Canada / Canada.ca</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/transport-canada/news/2026/08/government-of-canada-invests-over-235-million-to-strengthen-bc-airports-and-keep-communities-connected.html</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Contact the procurement offices of each of the six named BC airports directly; monitor BC Bid and each airport authority's local procurement portal for civil works ITTs expected to post within 30–60 days as airport authorities move from funding announcement to construction tender.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Transport Canada announced August 26, 2026 that over $23.5 million will fund critical infrastructure improvements at six BC airports through the Airports Capital Assistance Program; individual airport authorities will now procure civil and structural construction services locally.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -627,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -761,7 +1043,6 @@
           <t>jane\@example.com</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -775,6 +1056,144 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>Example row - delete before use</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Stuart McDonald</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Trekor Metals Limited (TSX: TKO)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Trekor Metals / GlobeNewswire</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/economy/articles/trekor-advances-environmental-assessment-yellowhead-123000463.html</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Reach out via Trekor's Vancouver investor relations contact (trekormetals.com) referencing the EAO Readiness Decision milestone; introduce heavy civil, site preparation, and transmission line capabilities relevant to the mine's new power line requirement; request a meeting ahead of formal RFQ release.</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>McDonald is the decision-maker behind the Yellowhead copper project, which received a positive BC EAO Readiness Decision on July 30, 2026 and is entering process planning for a 25-year, $47B-economic-output open-pit mine near Kamloops; he is actively advancing engineering studies and a summer 2026 drilling program and will soon be seeking civil engineering and mine infrastructure contractors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Catalin Kilofliski</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Canagold Resources Ltd. (TSX: CCM)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Newsfile Corp / Canagold Resources</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.newsfilecorp.com/release/295407/Canagold-New-Polaris-GoldAntimony-Project-Recognized-as-a-Priority-Project-by-British-Columbia</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Email Catalin directly at catalin@canagoldresources.com or call 604-685-9700; lead with northern BC remote construction logistics experience, Indigenous partnership credentials, and underground civil capability relevant to the coastal-mountain project site south of Atlin.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Kilofliski is driving the $757M New Polaris underground mine in northwest BC through BC EAO review after filing the EA application in April 2026 and securing BC priority-project status in May 2026; with over 25 years of executive leadership in BC mining and a 7,000-metre 2026 drill program underway, he is the key contact for early-stage civil, logistics, and underground construction pre-qualification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mark Liedemann</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Infrastructure BC</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ReNew Canada / Infrastructure BC</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.renewcanada.net/latest-edition-of-bc-major-infrastructure-projects-brochure-released/</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Download the Spring 2026 BC Major Infrastructure Projects Brochure from infrastructurebc.com; contact Infrastructure BC's business development team to register your firm's capabilities and request a market-sounding meeting ahead of the next project RFQ releases; attend the next Canadian Collaborative Contracts Conference event where Infrastructure BC presents.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Liedemann oversees BC's major public infrastructure procurement pipeline — including the Iona Island WWTP ($6B), Surrey-Langley SkyTrain ($6B), Fraser River Tunnel ($4.15B), and the Cowichan and Dawson Creek hospital redevelopments — and publishes the BC Major Infrastructure Projects Brochure that is the authoritative forward view for contractors; he is the gateway relationship for the province's $37.7B three-year capital program.</t>
         </is>
       </c>
     </row>

</xml_diff>